<commit_message>
Update roster: Operation Roster July2026 Version 3.xlsx
</commit_message>
<xml_diff>
--- a/rosters/.versions/2026-07/current.xlsx
+++ b/rosters/.versions/2026-07/current.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://omanair-my.sharepoint.com/personal/80235_hq_omanair_com/Documents/Desktop/Rosters/STAFF OPERATION SCHEDULE/Roster with 2 OFF/06July2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D3256F7B-B7F9-4266-85FE-800612D45F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2E930D9D-B943-4A2A-BBA5-12959476802B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{9736B67C-D61B-41E1-B07B-429B3D8AE9CC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="5" xr2:uid="{9736B67C-D61B-41E1-B07B-429B3D8AE9CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Setting " sheetId="1" state="hidden" r:id="rId1"/>
@@ -108,7 +108,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J10" authorId="0" shapeId="0" xr:uid="{426396D3-8A1C-44DA-A891-BB4A6D9F8F39}">
+    <comment ref="J10" authorId="0" shapeId="0" xr:uid="{43514C4B-EE7B-4EA4-8659-3CE9273213DF}">
       <text>
         <r>
           <rPr>
@@ -132,7 +132,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB10" authorId="0" shapeId="0" xr:uid="{C86AD1A7-BFA3-4B72-A33D-DFF1DBB266DE}">
+    <comment ref="AB10" authorId="0" shapeId="0" xr:uid="{4C490BD9-63D4-48AF-B7AD-D8D4C51F3C28}">
       <text>
         <r>
           <rPr>
@@ -156,7 +156,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI11" authorId="0" shapeId="0" xr:uid="{5D831B76-6760-4028-96FA-0877883C979A}">
+    <comment ref="AI11" authorId="0" shapeId="0" xr:uid="{16898DB3-D7F5-4A75-A8D9-8FD7C60743EE}">
       <text>
         <r>
           <rPr>
@@ -180,7 +180,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y12" authorId="0" shapeId="0" xr:uid="{9E7FA1D2-DA25-4971-AFAE-D0635C0CF5D4}">
+    <comment ref="Y12" authorId="0" shapeId="0" xr:uid="{7844651C-7414-4ACA-A710-6736176A919E}">
       <text>
         <r>
           <rPr>
@@ -204,7 +204,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z12" authorId="0" shapeId="0" xr:uid="{5B6EF41C-19BF-49FC-9D84-0BE498A43CAA}">
+    <comment ref="Z12" authorId="0" shapeId="0" xr:uid="{4B698108-387B-4D1B-939C-05520EAC4ED3}">
       <text>
         <r>
           <rPr>
@@ -228,7 +228,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L13" authorId="0" shapeId="0" xr:uid="{2310BEB2-1C39-4377-A8E0-32FB94C091B6}">
+    <comment ref="L13" authorId="0" shapeId="0" xr:uid="{0EAFB97E-76D4-4837-A12C-B01C3AF3E59F}">
       <text>
         <r>
           <rPr>
@@ -252,7 +252,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S13" authorId="0" shapeId="0" xr:uid="{E69A11E0-6461-4556-A65E-513DC626F312}">
+    <comment ref="S13" authorId="0" shapeId="0" xr:uid="{2E030B56-0810-41E5-86A1-34750762B611}">
       <text>
         <r>
           <rPr>
@@ -276,7 +276,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R15" authorId="0" shapeId="0" xr:uid="{23096079-B9AE-454B-AAF8-5CBF876D9B34}">
+    <comment ref="R15" authorId="0" shapeId="0" xr:uid="{C35E9700-14F0-4D7E-AEC4-B969D5B0DB12}">
       <text>
         <r>
           <rPr>
@@ -300,7 +300,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S15" authorId="0" shapeId="0" xr:uid="{18F2AFD5-FE29-4E2F-8326-24017F4EFEF4}">
+    <comment ref="S15" authorId="0" shapeId="0" xr:uid="{6B6B4202-608E-4612-AECE-FB56CCA02EFC}">
       <text>
         <r>
           <rPr>
@@ -324,7 +324,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L16" authorId="0" shapeId="0" xr:uid="{CD3913D8-04F9-4187-8CDB-165BB53A9F41}">
+    <comment ref="L16" authorId="0" shapeId="0" xr:uid="{173772C8-9BD0-420D-B7E4-09761F947A1B}">
       <text>
         <r>
           <rPr>
@@ -348,7 +348,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S16" authorId="0" shapeId="0" xr:uid="{6D81F792-D85E-4580-81F9-76D6D574BE11}">
+    <comment ref="S16" authorId="0" shapeId="0" xr:uid="{B50A7DCE-B1C6-46AC-AB55-161E56996110}">
       <text>
         <r>
           <rPr>
@@ -372,7 +372,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J17" authorId="0" shapeId="0" xr:uid="{CDC77B29-0880-49CA-A9F7-E4227F049950}">
+    <comment ref="J17" authorId="0" shapeId="0" xr:uid="{43896DD2-FA98-444E-B235-3A9476C1FD32}">
       <text>
         <r>
           <rPr>
@@ -396,7 +396,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y17" authorId="0" shapeId="0" xr:uid="{03EDD528-E546-47DE-9576-064ADDD3A6AE}">
+    <comment ref="Y17" authorId="0" shapeId="0" xr:uid="{6BA07AEE-72A7-4725-8E2F-D526530442FA}">
       <text>
         <r>
           <rPr>
@@ -420,7 +420,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z17" authorId="0" shapeId="0" xr:uid="{95AA8042-EDA4-4759-9E09-D262E5E0EDC1}">
+    <comment ref="Z17" authorId="0" shapeId="0" xr:uid="{A153B819-9BDA-452A-A39D-C619E420275A}">
       <text>
         <r>
           <rPr>
@@ -444,7 +444,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB18" authorId="0" shapeId="0" xr:uid="{36FF520A-0A51-4029-92DE-1CEEE31F279C}">
+    <comment ref="AB18" authorId="0" shapeId="0" xr:uid="{0A2BABB3-02FB-4793-9BA0-D0EF6EBF677E}">
       <text>
         <r>
           <rPr>
@@ -458,7 +458,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI18" authorId="0" shapeId="0" xr:uid="{54D8BC7D-8397-42C5-B4F2-F48B732236C2}">
+    <comment ref="AI18" authorId="0" shapeId="0" xr:uid="{0785E858-C063-446A-A795-99616BD8500B}">
       <text>
         <r>
           <rPr>
@@ -482,7 +482,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M19" authorId="0" shapeId="0" xr:uid="{A5AB5ED9-B40C-469E-B28B-FB6776D8BA1B}">
+    <comment ref="M19" authorId="0" shapeId="0" xr:uid="{3D1E6E42-7C02-4690-B52C-59A24153D806}">
       <text>
         <r>
           <rPr>
@@ -506,7 +506,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI20" authorId="0" shapeId="0" xr:uid="{EA1C19D4-D83A-4835-A169-E86FC6D26505}">
+    <comment ref="AI20" authorId="0" shapeId="0" xr:uid="{143FC73D-966B-4670-B651-97F8ADDC0024}">
       <text>
         <r>
           <rPr>
@@ -530,7 +530,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y22" authorId="0" shapeId="0" xr:uid="{980FA208-6709-4E0A-9F5D-4781064B2D8D}">
+    <comment ref="Y22" authorId="0" shapeId="0" xr:uid="{278E662D-14A8-48C2-B0B3-D133D89C7F74}">
       <text>
         <r>
           <rPr>
@@ -554,7 +554,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z22" authorId="0" shapeId="0" xr:uid="{39039648-FE63-443D-90E4-42245B92B064}">
+    <comment ref="Z22" authorId="0" shapeId="0" xr:uid="{668C575E-B9DF-472A-8145-2AAFD6251BD6}">
       <text>
         <r>
           <rPr>
@@ -578,7 +578,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S24" authorId="0" shapeId="0" xr:uid="{96F206AF-4395-47A7-88CE-199D87BB4551}">
+    <comment ref="S24" authorId="0" shapeId="0" xr:uid="{B46392B7-7812-4C1C-B207-7AA6242EF059}">
       <text>
         <r>
           <rPr>
@@ -602,7 +602,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y24" authorId="0" shapeId="0" xr:uid="{F1512EB0-0C72-48C8-A593-94FA91959EB7}">
+    <comment ref="Y24" authorId="0" shapeId="0" xr:uid="{EF943B50-C8E9-4DA4-B933-07287C9A118D}">
       <text>
         <r>
           <rPr>
@@ -626,7 +626,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE24" authorId="0" shapeId="0" xr:uid="{4498D380-7DF3-4E6F-A404-A7077C84644D}">
+    <comment ref="AE24" authorId="0" shapeId="0" xr:uid="{8B276A69-12A9-44F8-80C0-88E96BCFFE94}">
       <text>
         <r>
           <rPr>
@@ -650,7 +650,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J25" authorId="0" shapeId="0" xr:uid="{9DB44E84-7C77-44BC-80EE-80D31AF94351}">
+    <comment ref="J25" authorId="0" shapeId="0" xr:uid="{83648FF0-F726-4878-92A6-4C1668F85753}">
       <text>
         <r>
           <rPr>
@@ -674,7 +674,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB25" authorId="0" shapeId="0" xr:uid="{611C1897-A56C-49B6-A2D5-CACAACC42A1E}">
+    <comment ref="AB25" authorId="0" shapeId="0" xr:uid="{DCFAF17A-9921-4DD8-8EBA-14B0C4268272}">
       <text>
         <r>
           <rPr>
@@ -698,7 +698,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AC25" authorId="0" shapeId="0" xr:uid="{5709A706-8F81-491B-B46C-BA127E5B0FB1}">
+    <comment ref="AC25" authorId="0" shapeId="0" xr:uid="{CD61DD13-5CE0-4537-A04C-34337BA9986E}">
       <text>
         <r>
           <rPr>
@@ -722,7 +722,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AF25" authorId="0" shapeId="0" xr:uid="{E4D4B5D5-1F9C-47A2-AB9A-87EA4DE48F47}">
+    <comment ref="AF25" authorId="0" shapeId="0" xr:uid="{6B9C1DE6-34C3-477F-813F-AB9C9C1542EC}">
       <text>
         <r>
           <rPr>
@@ -746,7 +746,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J26" authorId="0" shapeId="0" xr:uid="{3448AF57-1FBE-4F76-98B4-105C931EC217}">
+    <comment ref="J26" authorId="0" shapeId="0" xr:uid="{2BC658BA-61B1-45AF-AA13-A7534379B5BE}">
       <text>
         <r>
           <rPr>
@@ -770,7 +770,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB26" authorId="0" shapeId="0" xr:uid="{541EC8EA-4205-40A5-B59F-7AE042B5D99A}">
+    <comment ref="AB26" authorId="0" shapeId="0" xr:uid="{C186C24C-4756-406A-92F9-8FE0B1BD649F}">
       <text>
         <r>
           <rPr>
@@ -794,7 +794,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB29" authorId="0" shapeId="0" xr:uid="{EF48A00C-927C-4402-A365-F29BD06AE603}">
+    <comment ref="AB29" authorId="0" shapeId="0" xr:uid="{4CAB269C-B845-43F1-8521-C25005672E20}">
       <text>
         <r>
           <rPr>
@@ -818,7 +818,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB33" authorId="0" shapeId="0" xr:uid="{E96EBEEA-2C0B-4E46-9386-EF4DAB9B6F25}">
+    <comment ref="AB33" authorId="0" shapeId="0" xr:uid="{18E5CBA1-0150-48D1-A6BE-4B3975A62B67}">
       <text>
         <r>
           <rPr>
@@ -842,7 +842,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB34" authorId="0" shapeId="0" xr:uid="{00045213-8A90-43C6-8219-5B549F94BAB2}">
+    <comment ref="AB34" authorId="0" shapeId="0" xr:uid="{79EE88A1-BE92-44B7-B54E-691C427BA81D}">
       <text>
         <r>
           <rPr>
@@ -866,7 +866,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB35" authorId="0" shapeId="0" xr:uid="{90E36C80-082F-4543-9567-77BEAD4581D9}">
+    <comment ref="AB35" authorId="0" shapeId="0" xr:uid="{CF041CF8-CC56-49A0-9D18-99D8972EF1FC}">
       <text>
         <r>
           <rPr>
@@ -890,7 +890,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L36" authorId="0" shapeId="0" xr:uid="{8DB04E09-CD91-4DCA-83B8-B90E300B8D9C}">
+    <comment ref="L36" authorId="0" shapeId="0" xr:uid="{45AE3C0B-7A46-46AE-9AA9-D609B8CB0010}">
       <text>
         <r>
           <rPr>
@@ -914,7 +914,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S36" authorId="0" shapeId="0" xr:uid="{2407BF5D-FCD8-4205-BC54-F50A201BDC3C}">
+    <comment ref="S36" authorId="0" shapeId="0" xr:uid="{AE8305EA-7DD0-4AA1-91A7-449E69BF4D2D}">
       <text>
         <r>
           <rPr>
@@ -938,7 +938,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N39" authorId="0" shapeId="0" xr:uid="{E28782D5-EB19-49D2-88D9-94A5D200F0F8}">
+    <comment ref="N39" authorId="0" shapeId="0" xr:uid="{B9D6C082-9E8C-4C12-98CD-D60C1BDFB4AE}">
       <text>
         <r>
           <rPr>
@@ -962,7 +962,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB40" authorId="0" shapeId="0" xr:uid="{E33ACD2A-020A-48AA-B925-69B9D5DF2B58}">
+    <comment ref="AB40" authorId="0" shapeId="0" xr:uid="{C65C1C97-2B3F-443B-BEFD-343A3AD541BF}">
       <text>
         <r>
           <rPr>
@@ -986,7 +986,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI41" authorId="0" shapeId="0" xr:uid="{AB261E19-BD15-4AB6-A9F4-222D27DB44DD}">
+    <comment ref="AI41" authorId="0" shapeId="0" xr:uid="{27E016D5-7D87-462C-96D9-021BF7DBB926}">
       <text>
         <r>
           <rPr>
@@ -1010,7 +1010,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH42" authorId="0" shapeId="0" xr:uid="{79611FE0-F581-460A-AE6F-0A8E14EBF267}">
+    <comment ref="AH42" authorId="0" shapeId="0" xr:uid="{D82244DE-86F9-44B4-B90C-74B3E78F8189}">
       <text>
         <r>
           <rPr>
@@ -1034,7 +1034,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M43" authorId="0" shapeId="0" xr:uid="{CA2A6E82-127E-46A7-8225-F7FD5E26B6BD}">
+    <comment ref="M43" authorId="0" shapeId="0" xr:uid="{26099D1E-1618-4E38-A917-C4DBA273DC49}">
       <text>
         <r>
           <rPr>
@@ -1058,7 +1058,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T43" authorId="0" shapeId="0" xr:uid="{7D3A2670-F674-4DB0-9DB3-71646A11EB21}">
+    <comment ref="T43" authorId="0" shapeId="0" xr:uid="{E8A3FB2D-5723-494C-A3EC-D9606A8C8DDB}">
       <text>
         <r>
           <rPr>
@@ -1082,7 +1082,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S44" authorId="0" shapeId="0" xr:uid="{647B5901-D8DE-4358-88AA-4A5D6D69BB70}">
+    <comment ref="S44" authorId="0" shapeId="0" xr:uid="{86EBE805-2D74-4928-9CFD-054724F22A9F}">
       <text>
         <r>
           <rPr>
@@ -1106,7 +1106,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB47" authorId="0" shapeId="0" xr:uid="{EF01B265-DF85-458F-9CB8-9A4086F39BDA}">
+    <comment ref="AB47" authorId="0" shapeId="0" xr:uid="{50E78CF5-3052-4584-9ACD-41F501C8C173}">
       <text>
         <r>
           <rPr>
@@ -1130,7 +1130,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI47" authorId="0" shapeId="0" xr:uid="{BC5C148B-6A26-49E9-9AC5-D0D984849258}">
+    <comment ref="AI47" authorId="0" shapeId="0" xr:uid="{2A023BCE-8B6D-4228-8FAF-D3CD5A217B10}">
       <text>
         <r>
           <rPr>
@@ -1154,7 +1154,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S50" authorId="0" shapeId="0" xr:uid="{EA0C5658-6083-4E36-A132-728886A10407}">
+    <comment ref="S50" authorId="0" shapeId="0" xr:uid="{A01DAA5E-C33C-42B5-8176-AE967693BC20}">
       <text>
         <r>
           <rPr>
@@ -1178,7 +1178,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI53" authorId="0" shapeId="0" xr:uid="{4593A513-FB3A-4180-8D99-BC92AB5FDE02}">
+    <comment ref="AI53" authorId="0" shapeId="0" xr:uid="{3A541D34-326D-4C0D-B64E-446146E80954}">
       <text>
         <r>
           <rPr>
@@ -1202,7 +1202,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S55" authorId="0" shapeId="0" xr:uid="{42490A06-BE85-4012-8A27-31013BE2A08A}">
+    <comment ref="S55" authorId="0" shapeId="0" xr:uid="{6EE19B44-EE8C-485E-9CF5-F9B9FE868434}">
       <text>
         <r>
           <rPr>
@@ -1226,7 +1226,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI56" authorId="0" shapeId="0" xr:uid="{D6ACD78F-D8D2-49C7-8AA9-961DAD73D64F}">
+    <comment ref="AI56" authorId="0" shapeId="0" xr:uid="{23FD1A43-613C-421D-8236-12BBE1F3099C}">
       <text>
         <r>
           <rPr>
@@ -1250,7 +1250,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y58" authorId="0" shapeId="0" xr:uid="{60ADD6EF-6E6A-4FCE-A60B-7D7E8E0DC4E4}">
+    <comment ref="Y58" authorId="0" shapeId="0" xr:uid="{46992F23-EFBA-436A-BB10-D37209948EFD}">
       <text>
         <r>
           <rPr>
@@ -1274,7 +1274,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z58" authorId="0" shapeId="0" xr:uid="{1638596E-17F5-40AD-B2A6-ED9DC6515F4B}">
+    <comment ref="Z58" authorId="0" shapeId="0" xr:uid="{64D90541-E0C0-4E13-AE54-F20742A3B939}">
       <text>
         <r>
           <rPr>
@@ -1298,7 +1298,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S61" authorId="0" shapeId="0" xr:uid="{6EDF3420-E170-47EE-91B4-0437EDD977AE}">
+    <comment ref="S61" authorId="0" shapeId="0" xr:uid="{9E944B94-2DFA-490E-B9CA-9EB29A031C7B}">
       <text>
         <r>
           <rPr>
@@ -1322,7 +1322,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI66" authorId="0" shapeId="0" xr:uid="{32E1F3BA-7F99-4DB2-9B11-4C6820B20446}">
+    <comment ref="AI66" authorId="0" shapeId="0" xr:uid="{342D5894-50BB-4901-AE96-8F886052826A}">
       <text>
         <r>
           <rPr>
@@ -1346,7 +1346,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG74" authorId="0" shapeId="0" xr:uid="{3761EC1E-57FE-4B2F-B1CF-473FA6CB4285}">
+    <comment ref="AG74" authorId="0" shapeId="0" xr:uid="{C3F9ECF9-7962-4685-9214-E6F8203D54E5}">
       <text>
         <r>
           <rPr>
@@ -4795,103 +4795,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="145">
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor auto="1"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="134">
     <dxf>
       <fill>
         <patternFill>
@@ -11986,26 +11890,26 @@
     <mergeCell ref="X4:Z4"/>
   </mergeCells>
   <conditionalFormatting sqref="E8:AI37 AK8:AN37 E39:AI42">
-    <cfRule type="expression" dxfId="144" priority="4">
+    <cfRule type="expression" dxfId="133" priority="4">
       <formula>LEFT(E8,1)="N"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="143" priority="5">
+    <cfRule type="expression" dxfId="132" priority="5">
       <formula>LEFT(E8,1)="A"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="142" priority="7">
+    <cfRule type="expression" dxfId="131" priority="7">
       <formula>LEFT(E8,1)="M"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="141" priority="8">
+    <cfRule type="expression" dxfId="130" priority="8">
       <formula>LEFT(E8,1)="D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E39:AI42 E8:AI37 AK8:AN37">
-    <cfRule type="expression" dxfId="140" priority="3">
+    <cfRule type="expression" dxfId="129" priority="3">
       <formula>LEFT(E8,1)="O"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E39:AI42">
-    <cfRule type="expression" dxfId="139" priority="1">
+    <cfRule type="expression" dxfId="128" priority="1">
       <formula>ISEVEN(ROW($E39))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13316,7 +13220,7 @@
         <v>209</v>
       </c>
       <c r="O13" s="110" t="s">
-        <v>209</v>
+        <v>237</v>
       </c>
       <c r="P13" s="110" t="s">
         <v>210</v>
@@ -13396,7 +13300,7 @@
       </c>
       <c r="AO13" s="48">
         <f t="shared" si="8"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AP13" s="48">
         <f t="shared" si="9"/>
@@ -14732,7 +14636,7 @@
         <v>210</v>
       </c>
       <c r="AJ24" s="94" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
       <c r="AL24" s="48">
         <f t="shared" si="10"/>
@@ -14744,7 +14648,7 @@
       </c>
       <c r="AN24" s="48">
         <f t="shared" si="12"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AO24" s="48">
         <f t="shared" si="13"/>
@@ -15461,7 +15365,7 @@
         <v>221</v>
       </c>
       <c r="AG30" s="83" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="AH30" s="83" t="s">
         <v>225</v>
@@ -15478,7 +15382,7 @@
       </c>
       <c r="AM30" s="48">
         <f t="shared" ref="AM30:AM73" si="16">COUNTIF($F30:$AJ30,"M*")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AN30" s="48">
         <f t="shared" ref="AN30:AN73" si="17">COUNTIF($F30:$AJ30,"A*")</f>
@@ -15486,7 +15390,7 @@
       </c>
       <c r="AO30" s="48">
         <f t="shared" ref="AO30:AO73" si="18">COUNTIF($F30:$AJ30,"N*")</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AP30" s="48">
         <f t="shared" ref="AP30:AP73" si="19">COUNTIF($F30:$AJ30,"O*")</f>
@@ -15836,7 +15740,7 @@
         <v>222</v>
       </c>
       <c r="AJ33" s="110" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="AL33" s="48">
         <f t="shared" si="15"/>
@@ -15844,11 +15748,11 @@
       </c>
       <c r="AM33" s="48">
         <f t="shared" si="16"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AN33" s="48">
         <f t="shared" si="17"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AO33" s="48">
         <f t="shared" si="18"/>
@@ -16276,10 +16180,10 @@
         <v>221</v>
       </c>
       <c r="T37" s="110" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="U37" s="110" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="V37" s="110" t="s">
         <v>210</v>
@@ -16340,7 +16244,7 @@
       </c>
       <c r="AO37" s="48">
         <f t="shared" si="18"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AP37" s="48">
         <f t="shared" si="19"/>
@@ -16648,13 +16552,13 @@
         <v>222</v>
       </c>
       <c r="V40" s="110" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="W40" s="110" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="X40" s="110" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="Y40" s="110" t="s">
         <v>210</v>
@@ -16698,7 +16602,7 @@
       </c>
       <c r="AM40" s="48">
         <f t="shared" si="16"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AN40" s="48">
         <f t="shared" si="17"/>
@@ -16706,7 +16610,7 @@
       </c>
       <c r="AO40" s="48">
         <f t="shared" si="18"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AP40" s="48">
         <f t="shared" si="19"/>
@@ -16981,7 +16885,7 @@
         <v>222</v>
       </c>
       <c r="K43" s="110" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="L43" s="110" t="s">
         <v>221</v>
@@ -17011,7 +16915,7 @@
         <v>126</v>
       </c>
       <c r="U43" s="110" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="V43" s="110" t="s">
         <v>210</v>
@@ -17064,7 +16968,7 @@
       </c>
       <c r="AM43" s="48">
         <f t="shared" si="16"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AN43" s="48">
         <f t="shared" si="17"/>
@@ -17072,7 +16976,7 @@
       </c>
       <c r="AO43" s="48">
         <f t="shared" si="18"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AP43" s="48">
         <f t="shared" si="19"/>
@@ -17862,7 +17766,7 @@
         <v>126</v>
       </c>
       <c r="T50" s="110" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="U50" s="110" t="s">
         <v>225</v>
@@ -17918,7 +17822,7 @@
       </c>
       <c r="AM50" s="48">
         <f t="shared" si="16"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AN50" s="48">
         <f t="shared" si="17"/>
@@ -17926,7 +17830,7 @@
       </c>
       <c r="AO50" s="48">
         <f t="shared" si="18"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AP50" s="48">
         <f t="shared" si="19"/>
@@ -18234,7 +18138,7 @@
         <v>222</v>
       </c>
       <c r="V53" s="110" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="W53" s="110" t="s">
         <v>221</v>
@@ -18284,11 +18188,11 @@
       </c>
       <c r="AM53" s="48">
         <f t="shared" si="16"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AN53" s="48">
         <f t="shared" si="17"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AO53" s="48">
         <f t="shared" si="18"/>
@@ -18597,7 +18501,7 @@
         <v>221</v>
       </c>
       <c r="U56" s="84" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="V56" s="84" t="s">
         <v>225</v>
@@ -18650,7 +18554,7 @@
       </c>
       <c r="AM56" s="48">
         <f t="shared" si="16"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AN56" s="48">
         <f t="shared" si="17"/>
@@ -18658,7 +18562,7 @@
       </c>
       <c r="AO56" s="48">
         <f t="shared" si="18"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AP56" s="48">
         <f t="shared" si="19"/>
@@ -21065,7 +20969,7 @@
       </c>
       <c r="K77" s="37">
         <f t="shared" si="25"/>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L77" s="37">
         <f t="shared" si="25"/>
@@ -21101,11 +21005,11 @@
       </c>
       <c r="T77" s="37">
         <f t="shared" si="25"/>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="U77" s="37">
         <f t="shared" si="25"/>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="V77" s="37">
         <f t="shared" si="25"/>
@@ -21113,7 +21017,7 @@
       </c>
       <c r="W77" s="37">
         <f t="shared" si="25"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="X77" s="37">
         <f t="shared" si="25"/>
@@ -21153,7 +21057,7 @@
       </c>
       <c r="AG77" s="37">
         <f t="shared" si="25"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AH77" s="37">
         <f t="shared" si="25"/>
@@ -21165,7 +21069,7 @@
       </c>
       <c r="AJ77" s="37">
         <f t="shared" si="25"/>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AL77" s="48">
         <f t="shared" si="24"/>
@@ -21260,7 +21164,7 @@
       </c>
       <c r="V78" s="37">
         <f t="shared" si="26"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="W78" s="37">
         <f t="shared" si="26"/>
@@ -21383,7 +21287,7 @@
       </c>
       <c r="O79" s="37">
         <f t="shared" si="27"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="P79" s="37">
         <f t="shared" si="27"/>
@@ -21407,7 +21311,7 @@
       </c>
       <c r="U79" s="37">
         <f t="shared" si="27"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="V79" s="37">
         <f t="shared" si="27"/>
@@ -21419,7 +21323,7 @@
       </c>
       <c r="X79" s="37">
         <f t="shared" si="27"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Y79" s="37">
         <f t="shared" si="27"/>
@@ -21455,7 +21359,7 @@
       </c>
       <c r="AG79" s="37">
         <f t="shared" si="27"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AH79" s="37">
         <f t="shared" si="27"/>
@@ -21971,7 +21875,7 @@
       </c>
       <c r="K83" s="50">
         <f t="shared" si="31"/>
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="L83" s="50">
         <f t="shared" si="31"/>
@@ -21987,7 +21891,7 @@
       </c>
       <c r="O83" s="50">
         <f t="shared" si="31"/>
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="P83" s="50">
         <f t="shared" si="31"/>
@@ -22007,23 +21911,23 @@
       </c>
       <c r="T83" s="50">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="U83" s="50">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="V83" s="50">
         <f t="shared" si="31"/>
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="W83" s="50">
         <f t="shared" si="31"/>
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="X83" s="50">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="Y83" s="50">
         <f t="shared" si="31"/>
@@ -22178,7 +22082,7 @@
       </c>
       <c r="K85" s="41">
         <f t="shared" si="32"/>
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L85" s="41">
         <f t="shared" si="32"/>
@@ -22194,7 +22098,7 @@
       </c>
       <c r="O85" s="41">
         <f t="shared" si="32"/>
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P85" s="41">
         <f t="shared" si="32"/>
@@ -22214,23 +22118,23 @@
       </c>
       <c r="T85" s="41">
         <f t="shared" si="32"/>
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="U85" s="41">
         <f t="shared" si="32"/>
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="V85" s="41">
         <f t="shared" si="32"/>
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="W85" s="41">
         <f t="shared" si="32"/>
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="X85" s="41">
         <f t="shared" si="32"/>
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Y85" s="41">
         <f t="shared" si="32"/>
@@ -22448,7 +22352,7 @@
       </c>
       <c r="K87" s="37">
         <f t="shared" si="33"/>
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="L87" s="37">
         <f t="shared" si="33"/>
@@ -22464,7 +22368,7 @@
       </c>
       <c r="O87" s="37">
         <f t="shared" si="33"/>
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P87" s="37">
         <f t="shared" si="33"/>
@@ -22484,23 +22388,23 @@
       </c>
       <c r="T87" s="37">
         <f t="shared" si="33"/>
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="U87" s="37">
         <f t="shared" si="33"/>
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="V87" s="37">
         <f t="shared" si="33"/>
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="W87" s="37">
         <f t="shared" si="33"/>
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="X87" s="37">
         <f t="shared" si="33"/>
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="Y87" s="37">
         <f t="shared" si="33"/>
@@ -22926,127 +22830,129 @@
     <mergeCell ref="C69:D69"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
+  <conditionalFormatting sqref="F5:AJ8">
+    <cfRule type="containsText" dxfId="127" priority="28" operator="containsText" text="ME06">
+      <formula>NOT(ISERROR(SEARCH("ME06",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="126" priority="29" operator="containsText" text="AE14">
+      <formula>NOT(ISERROR(SEARCH("AE14",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="125" priority="30" operator="containsText" text="ME07">
+      <formula>NOT(ISERROR(SEARCH("ME07",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="124" priority="31" operator="containsText" text="AE14">
+      <formula>NOT(ISERROR(SEARCH("AE14",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="123" priority="32" operator="containsText" text="ME06">
+      <formula>NOT(ISERROR(SEARCH("ME06",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="122" priority="33" operator="containsText" text="TR">
+      <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="121" priority="34" operator="containsText" text="MN06">
+      <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="120" priority="35" operator="containsText" text="AN13">
+      <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="119" priority="36" operator="containsText" text="OFF">
+      <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="118" priority="37" operator="containsText" text="ME07">
+      <formula>NOT(ISERROR(SEARCH("ME07",F5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F5:AJ8">
+    <cfRule type="containsText" dxfId="117" priority="27" operator="containsText" text="LV">
+      <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F62:AJ75">
-    <cfRule type="containsText" dxfId="36" priority="31" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="25" priority="20" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F62)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="35" priority="32" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="24" priority="21" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F62)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="34" priority="33" operator="containsText" text="ME06">
+    <cfRule type="containsText" dxfId="23" priority="22" operator="containsText" text="ME06">
       <formula>NOT(ISERROR(SEARCH("ME06",F62)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="33" priority="34" operator="containsText" text="AE14">
+    <cfRule type="containsText" dxfId="22" priority="23" operator="containsText" text="AE14">
       <formula>NOT(ISERROR(SEARCH("AE14",F62)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="32" priority="35" operator="containsText" text="NE22">
+    <cfRule type="containsText" dxfId="21" priority="24" operator="containsText" text="NE22">
       <formula>NOT(ISERROR(SEARCH("NE22",F62)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="31" priority="36" operator="containsText" text="AE14">
+    <cfRule type="containsText" dxfId="20" priority="25" operator="containsText" text="AE14">
       <formula>NOT(ISERROR(SEARCH("AE14",F62)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="30" priority="37" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="19" priority="26" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F62)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F30:AJ61">
-    <cfRule type="containsText" dxfId="29" priority="24" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="18" priority="13" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F30)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="28" priority="25" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="17" priority="14" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F30)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="27" priority="27" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="16" priority="16" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F30)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="26" priority="28" operator="containsText" text="NE22">
+    <cfRule type="containsText" dxfId="15" priority="17" operator="containsText" text="NE22">
       <formula>NOT(ISERROR(SEARCH("NE22",F30)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="25" priority="29" operator="containsText" text="AE14">
+    <cfRule type="containsText" dxfId="14" priority="18" operator="containsText" text="AE14">
       <formula>NOT(ISERROR(SEARCH("AE14",F30)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="24" priority="30" operator="containsText" text="ME06">
+    <cfRule type="containsText" dxfId="13" priority="19" operator="containsText" text="ME06">
       <formula>NOT(ISERROR(SEARCH("ME06",F30)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F61:AJ61">
-    <cfRule type="containsText" dxfId="23" priority="26" operator="containsText" text="ME12">
+    <cfRule type="containsText" dxfId="12" priority="15" operator="containsText" text="ME12">
       <formula>NOT(ISERROR(SEARCH("ME12",F61)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F15:AJ29">
-    <cfRule type="containsText" dxfId="22" priority="18" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="11" priority="7" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="21" priority="19" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="10" priority="8" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="20" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="9" priority="9" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="19" priority="21" operator="containsText" text="NE22">
+    <cfRule type="containsText" dxfId="8" priority="10" operator="containsText" text="NE22">
       <formula>NOT(ISERROR(SEARCH("NE22",F15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="22" operator="containsText" text="ME06">
+    <cfRule type="containsText" dxfId="7" priority="11" operator="containsText" text="ME06">
       <formula>NOT(ISERROR(SEARCH("ME06",F15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="23" operator="containsText" text="AE14">
+    <cfRule type="containsText" dxfId="6" priority="12" operator="containsText" text="AE14">
       <formula>NOT(ISERROR(SEARCH("AE14",F15)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F9:AJ14">
-    <cfRule type="containsText" dxfId="16" priority="12" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F9)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="13" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F9)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="14" operator="containsText" text="NN21">
+    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="NN21">
       <formula>NOT(ISERROR(SEARCH("NN21",F9)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="15" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="2" priority="4" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F9)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="16" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F9)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="17" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="0" priority="6" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F9)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F5:AJ8">
-    <cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="LV">
-      <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="ME06">
-      <formula>NOT(ISERROR(SEARCH("ME06",F5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="AE14">
-      <formula>NOT(ISERROR(SEARCH("AE14",F5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="4" operator="containsText" text="ME07">
-      <formula>NOT(ISERROR(SEARCH("ME07",F5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="5" operator="containsText" text="AE14">
-      <formula>NOT(ISERROR(SEARCH("AE14",F5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="ME06">
-      <formula>NOT(ISERROR(SEARCH("ME06",F5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="7" operator="containsText" text="TR">
-      <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="8" operator="containsText" text="MN06">
-      <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="9" operator="containsText" text="AN13">
-      <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="10" operator="containsText" text="OFF">
-      <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="11" operator="containsText" text="ME07">
-      <formula>NOT(ISERROR(SEARCH("ME07",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -25352,37 +25258,37 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ8">
-    <cfRule type="containsText" dxfId="108" priority="1" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="97" priority="1" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="107" priority="2" operator="containsText" text="ME06">
+    <cfRule type="containsText" dxfId="96" priority="2" operator="containsText" text="ME06">
       <formula>NOT(ISERROR(SEARCH("ME06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="106" priority="3" operator="containsText" text="AE14">
+    <cfRule type="containsText" dxfId="95" priority="3" operator="containsText" text="AE14">
       <formula>NOT(ISERROR(SEARCH("AE14",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="105" priority="4" operator="containsText" text="ME07">
+    <cfRule type="containsText" dxfId="94" priority="4" operator="containsText" text="ME07">
       <formula>NOT(ISERROR(SEARCH("ME07",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="104" priority="5" operator="containsText" text="AE14">
+    <cfRule type="containsText" dxfId="93" priority="5" operator="containsText" text="AE14">
       <formula>NOT(ISERROR(SEARCH("AE14",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="103" priority="6" operator="containsText" text="ME06">
+    <cfRule type="containsText" dxfId="92" priority="6" operator="containsText" text="ME06">
       <formula>NOT(ISERROR(SEARCH("ME06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="102" priority="7" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="91" priority="7" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="101" priority="8" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="90" priority="8" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="100" priority="9" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="89" priority="9" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="99" priority="10" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="88" priority="10" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="98" priority="11" operator="containsText" text="ME07">
+    <cfRule type="containsText" dxfId="87" priority="11" operator="containsText" text="ME07">
       <formula>NOT(ISERROR(SEARCH("ME07",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -26192,7 +26098,7 @@
         <v>209</v>
       </c>
       <c r="O9" s="107" t="s">
-        <v>209</v>
+        <v>237</v>
       </c>
       <c r="P9" s="107" t="s">
         <v>210</v>
@@ -26272,7 +26178,7 @@
       </c>
       <c r="AO9" s="48">
         <f t="shared" si="3"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AP9" s="48">
         <f t="shared" si="4"/>
@@ -26741,7 +26647,7 @@
       </c>
       <c r="O14" s="37">
         <f t="shared" si="7"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P14" s="37">
         <f t="shared" si="7"/>
@@ -27265,7 +27171,7 @@
       </c>
       <c r="O18" s="49">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P18" s="49">
         <f t="shared" si="11"/>
@@ -27432,7 +27338,7 @@
       </c>
       <c r="O20" s="41">
         <f t="shared" si="12"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P20" s="41">
         <f t="shared" si="12"/>
@@ -27662,7 +27568,7 @@
       </c>
       <c r="O22" s="37">
         <f t="shared" si="13"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P22" s="37">
         <f t="shared" si="13"/>
@@ -27942,22 +27848,22 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ10">
-    <cfRule type="containsText" dxfId="97" priority="1" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="86" priority="1" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="96" priority="2" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="85" priority="2" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="95" priority="3" operator="containsText" text="NN21">
+    <cfRule type="containsText" dxfId="84" priority="3" operator="containsText" text="NN21">
       <formula>NOT(ISERROR(SEARCH("NN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="94" priority="4" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="83" priority="4" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="93" priority="5" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="82" priority="5" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="92" priority="6" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="81" priority="6" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -29437,7 +29343,7 @@
         <v>210</v>
       </c>
       <c r="AJ14" s="94" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
       <c r="AL14" s="48">
         <f t="shared" si="0"/>
@@ -29449,7 +29355,7 @@
       </c>
       <c r="AN14" s="48">
         <f t="shared" si="2"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AO14" s="48">
         <f t="shared" si="3"/>
@@ -30363,7 +30269,7 @@
       </c>
       <c r="AJ22" s="37">
         <f t="shared" si="6"/>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="2:42" ht="18.75" x14ac:dyDescent="0.3">
@@ -31476,22 +31382,22 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ19">
-    <cfRule type="containsText" dxfId="91" priority="1" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="80" priority="1" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="90" priority="2" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="79" priority="2" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="89" priority="3" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="78" priority="3" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="88" priority="4" operator="containsText" text="NE22">
+    <cfRule type="containsText" dxfId="77" priority="4" operator="containsText" text="NE22">
       <formula>NOT(ISERROR(SEARCH("NE22",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="87" priority="5" operator="containsText" text="ME06">
+    <cfRule type="containsText" dxfId="76" priority="5" operator="containsText" text="ME06">
       <formula>NOT(ISERROR(SEARCH("ME06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="86" priority="6" operator="containsText" text="AE14">
+    <cfRule type="containsText" dxfId="75" priority="6" operator="containsText" text="AE14">
       <formula>NOT(ISERROR(SEARCH("AE14",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -31867,7 +31773,7 @@
         <v>221</v>
       </c>
       <c r="AG5" s="83" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="AH5" s="83" t="s">
         <v>225</v>
@@ -31884,7 +31790,7 @@
       </c>
       <c r="AM5" s="48">
         <f t="shared" ref="AM5:AM36" si="1">COUNTIF($F5:$AJ5,"M*")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AN5" s="48">
         <f t="shared" ref="AN5:AN36" si="2">COUNTIF($F5:$AJ5,"A*")</f>
@@ -31892,7 +31798,7 @@
       </c>
       <c r="AO5" s="48">
         <f t="shared" ref="AO5:AO36" si="3">COUNTIF($F5:$AJ5,"N*")</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AP5" s="48">
         <f t="shared" ref="AP5:AP36" si="4">COUNTIF($F5:$AJ5,"O*")</f>
@@ -32242,7 +32148,7 @@
         <v>222</v>
       </c>
       <c r="AJ8" s="103" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="AL8" s="48">
         <f t="shared" si="0"/>
@@ -32250,11 +32156,11 @@
       </c>
       <c r="AM8" s="48">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AN8" s="48">
         <f t="shared" si="2"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AO8" s="48">
         <f t="shared" si="3"/>
@@ -32682,10 +32588,10 @@
         <v>221</v>
       </c>
       <c r="T12" s="103" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="U12" s="103" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="V12" s="103" t="s">
         <v>210</v>
@@ -32746,7 +32652,7 @@
       </c>
       <c r="AO12" s="48">
         <f t="shared" si="3"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AP12" s="48">
         <f t="shared" si="4"/>
@@ -33054,13 +32960,13 @@
         <v>222</v>
       </c>
       <c r="V15" s="103" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="W15" s="103" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="X15" s="103" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="Y15" s="103" t="s">
         <v>210</v>
@@ -33104,7 +33010,7 @@
       </c>
       <c r="AM15" s="48">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AN15" s="48">
         <f t="shared" si="2"/>
@@ -33112,7 +33018,7 @@
       </c>
       <c r="AO15" s="48">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AP15" s="48">
         <f t="shared" si="4"/>
@@ -33387,7 +33293,7 @@
         <v>222</v>
       </c>
       <c r="K18" s="103" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="L18" s="103" t="s">
         <v>221</v>
@@ -33417,7 +33323,7 @@
         <v>126</v>
       </c>
       <c r="U18" s="103" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="V18" s="103" t="s">
         <v>210</v>
@@ -33470,7 +33376,7 @@
       </c>
       <c r="AM18" s="48">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AN18" s="48">
         <f t="shared" si="2"/>
@@ -33478,7 +33384,7 @@
       </c>
       <c r="AO18" s="48">
         <f t="shared" si="3"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AP18" s="48">
         <f t="shared" si="4"/>
@@ -34268,7 +34174,7 @@
         <v>126</v>
       </c>
       <c r="T25" s="103" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="U25" s="103" t="s">
         <v>225</v>
@@ -34324,7 +34230,7 @@
       </c>
       <c r="AM25" s="48">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AN25" s="48">
         <f t="shared" si="2"/>
@@ -34332,7 +34238,7 @@
       </c>
       <c r="AO25" s="48">
         <f t="shared" si="3"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AP25" s="48">
         <f t="shared" si="4"/>
@@ -34640,7 +34546,7 @@
         <v>222</v>
       </c>
       <c r="V28" s="103" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="W28" s="103" t="s">
         <v>221</v>
@@ -34690,11 +34596,11 @@
       </c>
       <c r="AM28" s="48">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AN28" s="48">
         <f t="shared" si="2"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AO28" s="48">
         <f t="shared" si="3"/>
@@ -35003,7 +34909,7 @@
         <v>221</v>
       </c>
       <c r="U31" s="84" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="V31" s="84" t="s">
         <v>225</v>
@@ -35056,7 +34962,7 @@
       </c>
       <c r="AM31" s="48">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AN31" s="48">
         <f t="shared" si="2"/>
@@ -35064,7 +34970,7 @@
       </c>
       <c r="AO31" s="48">
         <f t="shared" si="3"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AP31" s="48">
         <f t="shared" si="4"/>
@@ -35743,7 +35649,7 @@
       </c>
       <c r="K38" s="37">
         <f t="shared" si="5"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L38" s="37">
         <f t="shared" si="5"/>
@@ -35779,11 +35685,11 @@
       </c>
       <c r="T38" s="37">
         <f t="shared" si="5"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U38" s="37">
         <f t="shared" si="5"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V38" s="37">
         <f t="shared" si="5"/>
@@ -35791,7 +35697,7 @@
       </c>
       <c r="W38" s="37">
         <f t="shared" si="5"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X38" s="37">
         <f t="shared" si="5"/>
@@ -35831,7 +35737,7 @@
       </c>
       <c r="AG38" s="37">
         <f t="shared" si="5"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AH38" s="37">
         <f t="shared" si="5"/>
@@ -35843,7 +35749,7 @@
       </c>
       <c r="AJ38" s="37">
         <f t="shared" si="5"/>
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" spans="2:42" ht="18.75" x14ac:dyDescent="0.3">
@@ -35918,7 +35824,7 @@
       </c>
       <c r="V39" s="37">
         <f t="shared" si="6"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W39" s="37">
         <f t="shared" si="6"/>
@@ -35974,7 +35880,7 @@
       </c>
       <c r="AJ39" s="37">
         <f t="shared" si="6"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40" spans="2:42" ht="18.75" x14ac:dyDescent="0.3">
@@ -36045,7 +35951,7 @@
       </c>
       <c r="U40" s="37">
         <f t="shared" si="7"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V40" s="37">
         <f t="shared" si="7"/>
@@ -36057,7 +35963,7 @@
       </c>
       <c r="X40" s="37">
         <f t="shared" si="7"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Y40" s="37">
         <f t="shared" si="7"/>
@@ -36093,7 +35999,7 @@
       </c>
       <c r="AG40" s="37">
         <f t="shared" si="7"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AH40" s="37">
         <f t="shared" si="7"/>
@@ -36529,7 +36435,7 @@
       </c>
       <c r="K44" s="50">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="L44" s="50">
         <f t="shared" si="11"/>
@@ -36565,23 +36471,23 @@
       </c>
       <c r="T44" s="50">
         <f t="shared" si="11"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U44" s="50">
         <f t="shared" si="11"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="V44" s="50">
         <f t="shared" si="11"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W44" s="50">
         <f t="shared" si="11"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X44" s="50">
         <f t="shared" si="11"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Y44" s="50">
         <f t="shared" si="11"/>
@@ -36696,7 +36602,7 @@
       </c>
       <c r="K46" s="41">
         <f t="shared" si="12"/>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L46" s="41">
         <f t="shared" si="12"/>
@@ -36732,23 +36638,23 @@
       </c>
       <c r="T46" s="41">
         <f t="shared" si="12"/>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="U46" s="41">
         <f t="shared" si="12"/>
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="V46" s="41">
         <f t="shared" si="12"/>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="W46" s="41">
         <f t="shared" si="12"/>
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="X46" s="41">
         <f t="shared" si="12"/>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Y46" s="41">
         <f t="shared" si="12"/>
@@ -36926,7 +36832,7 @@
       </c>
       <c r="K48" s="37">
         <f t="shared" si="13"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L48" s="37">
         <f t="shared" si="13"/>
@@ -36962,23 +36868,23 @@
       </c>
       <c r="T48" s="37">
         <f t="shared" si="13"/>
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="U48" s="37">
         <f t="shared" si="13"/>
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="V48" s="37">
         <f t="shared" si="13"/>
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="W48" s="37">
         <f t="shared" si="13"/>
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="X48" s="37">
         <f t="shared" si="13"/>
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="Y48" s="37">
         <f t="shared" si="13"/>
@@ -37240,27 +37146,27 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ36">
-    <cfRule type="containsText" dxfId="85" priority="1" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="74" priority="1" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="84" priority="2" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="73" priority="2" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="83" priority="4" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="72" priority="4" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="82" priority="5" operator="containsText" text="NE22">
+    <cfRule type="containsText" dxfId="71" priority="5" operator="containsText" text="NE22">
       <formula>NOT(ISERROR(SEARCH("NE22",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="81" priority="6" operator="containsText" text="AE14">
+    <cfRule type="containsText" dxfId="70" priority="6" operator="containsText" text="AE14">
       <formula>NOT(ISERROR(SEARCH("AE14",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="80" priority="7" operator="containsText" text="ME06">
+    <cfRule type="containsText" dxfId="69" priority="7" operator="containsText" text="ME06">
       <formula>NOT(ISERROR(SEARCH("ME06",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F36:AJ36">
-    <cfRule type="containsText" dxfId="79" priority="3" operator="containsText" text="ME12">
+    <cfRule type="containsText" dxfId="68" priority="3" operator="containsText" text="ME12">
       <formula>NOT(ISERROR(SEARCH("ME12",F36)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -40792,25 +40698,25 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ18">
-    <cfRule type="containsText" dxfId="78" priority="1" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="67" priority="1" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="77" priority="2" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="66" priority="2" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="76" priority="3" operator="containsText" text="ME06">
+    <cfRule type="containsText" dxfId="65" priority="3" operator="containsText" text="ME06">
       <formula>NOT(ISERROR(SEARCH("ME06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="75" priority="4" operator="containsText" text="AE14">
+    <cfRule type="containsText" dxfId="64" priority="4" operator="containsText" text="AE14">
       <formula>NOT(ISERROR(SEARCH("AE14",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="74" priority="5" operator="containsText" text="NE22">
+    <cfRule type="containsText" dxfId="63" priority="5" operator="containsText" text="NE22">
       <formula>NOT(ISERROR(SEARCH("NE22",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="73" priority="6" operator="containsText" text="AE14">
+    <cfRule type="containsText" dxfId="62" priority="6" operator="containsText" text="AE14">
       <formula>NOT(ISERROR(SEARCH("AE14",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="72" priority="7" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="61" priority="7" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -43585,117 +43491,117 @@
     <mergeCell ref="B8:C8"/>
   </mergeCells>
   <conditionalFormatting sqref="E5:AH10">
-    <cfRule type="containsText" dxfId="71" priority="23" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="60" priority="23" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="70" priority="24" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="59" priority="24" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="69" priority="25" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="58" priority="25" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="68" priority="26" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="57" priority="26" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="67" priority="27" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="56" priority="27" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="66" priority="28" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="55" priority="28" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="65" priority="29" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="54" priority="29" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="64" priority="30" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="53" priority="30" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E5:AH15">
-    <cfRule type="containsText" dxfId="63" priority="19" operator="containsText" text="A">
+    <cfRule type="containsText" dxfId="52" priority="19" operator="containsText" text="A">
       <formula>NOT(ISERROR(SEARCH("A",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="62" priority="5" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="51" priority="5" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11:AH15">
-    <cfRule type="containsText" dxfId="61" priority="16" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="50" priority="16" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="60" priority="17" operator="containsText" text="O">
+    <cfRule type="containsText" dxfId="49" priority="17" operator="containsText" text="O">
       <formula>NOT(ISERROR(SEARCH("O",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="59" priority="18" operator="containsText" text="N">
+    <cfRule type="containsText" dxfId="48" priority="18" operator="containsText" text="N">
       <formula>NOT(ISERROR(SEARCH("N",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="58" priority="6" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="47" priority="6" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="57" priority="7" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="46" priority="7" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="56" priority="8" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="45" priority="8" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="55" priority="9" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="44" priority="9" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="54" priority="10" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="43" priority="10" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="53" priority="11" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="42" priority="11" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="52" priority="12" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="41" priority="12" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="51" priority="13" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="40" priority="13" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="50" priority="14" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="39" priority="14" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="49" priority="15" operator="containsText" text="STA">
+    <cfRule type="containsText" dxfId="38" priority="15" operator="containsText" text="STA">
       <formula>NOT(ISERROR(SEARCH("STA",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="48" priority="20" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="37" priority="20" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E11)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E5:AI15">
-    <cfRule type="containsText" dxfId="47" priority="3" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="36" priority="3" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="46" priority="4" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="35" priority="4" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="45" priority="1" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="34" priority="1" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="44" priority="2" operator="containsText" text="STA">
+    <cfRule type="containsText" dxfId="33" priority="2" operator="containsText" text="STA">
       <formula>NOT(ISERROR(SEARCH("STA",E5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5:AH5 E6:AH10">
-    <cfRule type="containsText" dxfId="43" priority="31" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="32" priority="31" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="42" priority="32" operator="containsText" text="STA">
+    <cfRule type="containsText" dxfId="31" priority="32" operator="containsText" text="STA">
       <formula>NOT(ISERROR(SEARCH("STA",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="41" priority="33" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="30" priority="33" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="40" priority="34" operator="containsText" text="O">
+    <cfRule type="containsText" dxfId="29" priority="34" operator="containsText" text="O">
       <formula>NOT(ISERROR(SEARCH("O",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="39" priority="35" operator="containsText" text="N">
+    <cfRule type="containsText" dxfId="28" priority="35" operator="containsText" text="N">
       <formula>NOT(ISERROR(SEARCH("N",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="38" priority="36" operator="containsText" text="A">
+    <cfRule type="containsText" dxfId="27" priority="36" operator="containsText" text="A">
       <formula>NOT(ISERROR(SEARCH("A",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="37" priority="37" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="26" priority="37" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -43735,6 +43641,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_activity xmlns="0ecd8b7c-869e-4f04-a6a3-066c3c63b311" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="مستند" ma:contentTypeID="0x01010053585A714B17B949862FA1B71BD97610" ma:contentTypeVersion="20" ma:contentTypeDescription="إنشاء مستند جديد." ma:contentTypeScope="" ma:versionID="dd8bd6d392f178541f6ccf1c351709a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns3="f1e9c892-1499-41bb-8a64-60ef909d8682" xmlns:ns4="0ecd8b7c-869e-4f04-a6a3-066c3c63b311" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9f246d41c9a2b9a4922388dcb99eeb28" ns1:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -44004,26 +43929,33 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7131BC6-00FD-4253-878E-994124306B86}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_activity xmlns="0ecd8b7c-869e-4f04-a6a3-066c3c63b311" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04335F04-3ECE-4043-846B-35335B1D83ED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="0ecd8b7c-869e-4f04-a6a3-066c3c63b311"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="f1e9c892-1499-41bb-8a64-60ef909d8682"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57D06F05-5672-4668-89C3-4F6754D4BC82}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -44043,32 +43975,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7131BC6-00FD-4253-878E-994124306B86}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04335F04-3ECE-4043-846B-35335B1D83ED}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="0ecd8b7c-869e-4f04-a6a3-066c3c63b311"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="f1e9c892-1499-41bb-8a64-60ef909d8682"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{456ceee3-7fed-44e8-a399-cd4111988137}" enabled="0" method="" siteId="{456ceee3-7fed-44e8-a399-cd4111988137}" removed="1"/>

</xml_diff>